<commit_message>
Review workbooks: wrap the structure cells; re-export the WDS Point Analysis PDF (EPMA v88)
- Structure columns (procedure and session) now wrap, so longer instructions are no longer cut off
- WDS Point Analysis PDF re-exported from the current workbook: Instructions tab plus the EPMA TAPP table

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TAPPs for review/EPMA_TAPP_v88_Review_Workbook.xlsx
+++ b/TAPPs for review/EPMA_TAPP_v88_Review_Workbook.xlsx
@@ -1549,7 +1549,7 @@
           <t>EML-EPMA-CC v2, EPMA-WDS+EDS major and minor elements in carbonaceous-chondrite silicates, oxides, sulfides, phosphates and carbonates</t>
         </is>
       </c>
-      <c r="F3" s="27" t="inlineStr">
+      <c r="F3" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -1569,7 +1569,7 @@
           <t>— Set by registration requirements; no review needed</t>
         </is>
       </c>
-      <c r="J3" s="27" t="inlineStr">
+      <c r="J3" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -1637,7 +1637,7 @@
           <t>EPMA-WDS+EDS (combines wavelength-dispersive and energy-dispersive spectrometry)</t>
         </is>
       </c>
-      <c r="F4" s="27" t="inlineStr">
+      <c r="F4" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -1657,7 +1657,7 @@
           <t>— Set by registration requirements; no review needed</t>
         </is>
       </c>
-      <c r="J4" s="27" t="inlineStr">
+      <c r="J4" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -1725,7 +1725,7 @@
           <t>Example Microanalysis Laboratory</t>
         </is>
       </c>
-      <c r="F5" s="27" t="inlineStr">
+      <c r="F5" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -1745,7 +1745,7 @@
           <t>— Set by registration requirements; no review needed</t>
         </is>
       </c>
-      <c r="J5" s="27" t="inlineStr">
+      <c r="J5" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -1813,7 +1813,7 @@
           <t>Example Microanalysis Laboratory</t>
         </is>
       </c>
-      <c r="F6" s="27" t="inlineStr">
+      <c r="F6" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -1833,7 +1833,7 @@
           <t>— Set by registration requirements; no review needed</t>
         </is>
       </c>
-      <c r="J6" s="27" t="inlineStr">
+      <c r="J6" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -1901,7 +1901,7 @@
           <t>https://ror.org/0example00</t>
         </is>
       </c>
-      <c r="F7" s="27" t="inlineStr">
+      <c r="F7" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -1921,7 +1921,7 @@
           <t>— Set by registration requirements; no review needed</t>
         </is>
       </c>
-      <c r="J7" s="27" t="inlineStr">
+      <c r="J7" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -1989,7 +1989,7 @@
           <t>January 2025</t>
         </is>
       </c>
-      <c r="F8" s="27" t="inlineStr">
+      <c r="F8" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -2009,7 +2009,7 @@
           <t>— Set by registration requirements; no review needed</t>
         </is>
       </c>
-      <c r="J8" s="27" t="inlineStr">
+      <c r="J8" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -2077,7 +2077,7 @@
           <t>Example Agency award EX-INST-0001 (instrument); award EX-DEV-0002 (procedure development)</t>
         </is>
       </c>
-      <c r="F9" s="27" t="inlineStr">
+      <c r="F9" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -2097,7 +2097,7 @@
           <t>— Set by registration requirements; no review needed</t>
         </is>
       </c>
-      <c r="J9" s="27" t="inlineStr">
+      <c r="J9" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -2165,7 +2165,7 @@
           <t>Example et al. (2025), doi:10.0000/example.2025.001</t>
         </is>
       </c>
-      <c r="F10" s="27" t="inlineStr">
+      <c r="F10" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -2185,7 +2185,7 @@
           <t>— Set by registration requirements; no review needed</t>
         </is>
       </c>
-      <c r="J10" s="27" t="inlineStr">
+      <c r="J10" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -2253,7 +2253,7 @@
           <t>doi:10.0000/example.epma-cc.v2</t>
         </is>
       </c>
-      <c r="F11" s="27" t="inlineStr">
+      <c r="F11" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2273,7 +2273,7 @@
           <t>— Set by registration requirements; no review needed</t>
         </is>
       </c>
-      <c r="J11" s="27" t="inlineStr">
+      <c r="J11" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -2341,7 +2341,7 @@
           <t>EML-2026-0412-A</t>
         </is>
       </c>
-      <c r="F12" s="27" t="inlineStr">
+      <c r="F12" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2361,7 +2361,7 @@
           <t>— Set by registration requirements; no review needed</t>
         </is>
       </c>
-      <c r="J12" s="27" t="inlineStr">
+      <c r="J12" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -2429,7 +2429,7 @@
           <t>Analyst A (ORCID 0000-0000-0000-0000)</t>
         </is>
       </c>
-      <c r="F13" s="27" t="inlineStr">
+      <c r="F13" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2449,7 +2449,7 @@
           <t>— Set by registration requirements; no review needed</t>
         </is>
       </c>
-      <c r="J13" s="27" t="inlineStr">
+      <c r="J13" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -2517,7 +2517,7 @@
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="F14" s="27" t="inlineStr">
+      <c r="F14" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2537,7 +2537,7 @@
           <t>— Set by registration requirements; no review needed</t>
         </is>
       </c>
-      <c r="J14" s="27" t="inlineStr">
+      <c r="J14" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -2605,7 +2605,7 @@
           <t>2026-04-14</t>
         </is>
       </c>
-      <c r="F15" s="27" t="inlineStr">
+      <c r="F15" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2625,7 +2625,7 @@
           <t>— Set by registration requirements; no review needed</t>
         </is>
       </c>
-      <c r="J15" s="27" t="inlineStr">
+      <c r="J15" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -2693,7 +2693,7 @@
           <t>Example Agency award EX-SCI-0003</t>
         </is>
       </c>
-      <c r="F16" s="27" t="inlineStr">
+      <c r="F16" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2713,7 +2713,7 @@
           <t>— Set by registration requirements; no review needed</t>
         </is>
       </c>
-      <c r="J16" s="27" t="inlineStr">
+      <c r="J16" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -2777,7 +2777,7 @@
           <t>SEM; NanoSIMS (oxygen isotopes of carbonates, Example Isotope Laboratory)</t>
         </is>
       </c>
-      <c r="F17" s="27" t="inlineStr">
+      <c r="F17" s="30" t="inlineStr">
         <is>
           <t>Give one or more values for the procedure.</t>
         </is>
@@ -2789,7 +2789,7 @@
         </is>
       </c>
       <c r="I17" s="38" t="n"/>
-      <c r="J17" s="27" t="inlineStr">
+      <c r="J17" s="30" t="inlineStr">
         <is>
           <t>Give one or more values for the session.</t>
         </is>
@@ -2845,7 +2845,7 @@
           <t>EPMA carbonate compositions select the matrix-matched reference material for the NanoSIMS mass-fractionation correction; SEM first, EPMA next (non-destructive), NanoSIMS last (sputtering destroys the analysed volume)</t>
         </is>
       </c>
-      <c r="F18" s="27" t="inlineStr">
+      <c r="F18" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -2857,7 +2857,7 @@
         </is>
       </c>
       <c r="I18" s="38" t="n"/>
-      <c r="J18" s="27" t="inlineStr">
+      <c r="J18" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -2913,7 +2913,7 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="F19" s="27" t="inlineStr">
+      <c r="F19" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2925,7 +2925,7 @@
         </is>
       </c>
       <c r="I19" s="38" t="n"/>
-      <c r="J19" s="27" t="inlineStr">
+      <c r="J19" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -2981,7 +2981,7 @@
           <t>same submission</t>
         </is>
       </c>
-      <c r="F20" s="27" t="inlineStr">
+      <c r="F20" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="I20" s="38" t="n"/>
-      <c r="J20" s="27" t="inlineStr">
+      <c r="J20" s="30" t="inlineStr">
         <is>
           <t>Give one or more values for the session.</t>
         </is>
@@ -3077,7 +3077,7 @@
           <t>Silicate mineral (olivine, pyroxene); oxide (magnetite, chromite, ilmenite); sulfide (pyrrhotite, pentlandite); phosphate (apatite, merrillite); carbonate (calcite, dolomite, breunnerite), in carbonaceous-chondrite material</t>
         </is>
       </c>
-      <c r="F23" s="27" t="inlineStr">
+      <c r="F23" s="30" t="inlineStr">
         <is>
           <t>List the material types the procedure is designed to analyse.</t>
         </is>
@@ -3089,7 +3089,7 @@
         </is>
       </c>
       <c r="I23" s="38" t="n"/>
-      <c r="J23" s="27" t="inlineStr">
+      <c r="J23" s="30" t="inlineStr">
         <is>
           <t>List the material types the procedure is designed to analyse.</t>
         </is>
@@ -3145,7 +3145,7 @@
           <t>Epoxy mount, dry-polished with diamond to 0.25 µm, carbon coated to 20 nm, for EX-CC-01; the same, plus Ar-ion polishing after the final diamond step, for EX-CC-02</t>
         </is>
       </c>
-      <c r="F24" s="27" t="inlineStr">
+      <c r="F24" s="30" t="inlineStr">
         <is>
           <t>Give one value; each "Sample Name" entry in a session inherits it.</t>
         </is>
@@ -3157,7 +3157,7 @@
         </is>
       </c>
       <c r="I24" s="38" t="n"/>
-      <c r="J24" s="27" t="inlineStr">
+      <c r="J24" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Sample Name".</t>
         </is>
@@ -3213,7 +3213,7 @@
           <t>EX-CC-01; EX-CC-02</t>
         </is>
       </c>
-      <c r="F25" s="27" t="inlineStr">
+      <c r="F25" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3225,7 +3225,7 @@
         </is>
       </c>
       <c r="I25" s="38" t="n"/>
-      <c r="J25" s="27" t="inlineStr">
+      <c r="J25" s="30" t="inlineStr">
         <is>
           <t>List every sample analysed in the session.</t>
         </is>
@@ -3281,7 +3281,7 @@
           <t>Analysis point, labelled by particle and point number; each X-ray map is one result for its mapped area</t>
         </is>
       </c>
-      <c r="F26" s="27" t="inlineStr">
+      <c r="F26" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -3293,7 +3293,7 @@
         </is>
       </c>
       <c r="I26" s="38" t="n"/>
-      <c r="J26" s="27" t="inlineStr">
+      <c r="J26" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -3349,7 +3349,7 @@
           <t>P1-01–P1-12, P2-01–P2-11, P3-01–P3-06 and map M1 for EX-CC-01; P1-01–P1-16, P2-01–P2-08 and map M2 for EX-CC-02</t>
         </is>
       </c>
-      <c r="F27" s="27" t="inlineStr">
+      <c r="F27" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3361,7 +3361,7 @@
         </is>
       </c>
       <c r="I27" s="38" t="n"/>
-      <c r="J27" s="27" t="inlineStr">
+      <c r="J27" s="30" t="inlineStr">
         <is>
           <t>For each "Sample Name", list the analysis points analysed in it.</t>
         </is>
@@ -3417,7 +3417,7 @@
           <t>Silicate mineral for P1-01–P1-12, oxide for P2-01–P2-06, sulfide for P2-07–P2-11, phosphate for P3-01–P3-06 (EX-CC-01); carbonate for P1-01–P1-16, silicate mineral for P2-01–P2-08 (EX-CC-02)</t>
         </is>
       </c>
-      <c r="F28" s="27" t="inlineStr">
+      <c r="F28" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3429,7 +3429,7 @@
         </is>
       </c>
       <c r="I28" s="38" t="n"/>
-      <c r="J28" s="27" t="inlineStr">
+      <c r="J28" s="30" t="inlineStr">
         <is>
           <t>For each "Sample Name", give one value for each of its "Sampling Unit Name" entries.</t>
         </is>
@@ -3485,7 +3485,7 @@
           <t>IGSN:EXAMPLE0001 for EX-CC-01; IGSN:EXAMPLE0002 for EX-CC-02</t>
         </is>
       </c>
-      <c r="F29" s="27" t="inlineStr">
+      <c r="F29" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3497,7 +3497,7 @@
         </is>
       </c>
       <c r="I29" s="38" t="n"/>
-      <c r="J29" s="27" t="inlineStr">
+      <c r="J29" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Sample Name".</t>
         </is>
@@ -3553,7 +3553,7 @@
           <t>Grains at least 5 µm across (10 µm for phosphates and carbonates); at least 3 µm from boundaries, cracks and inclusions in BSE (5 µm for defocused or rastered beams); phase confirmed from its EDS spectrum first; map areas include every target phase in a particle</t>
         </is>
       </c>
-      <c r="F30" s="27" t="inlineStr">
+      <c r="F30" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -3565,7 +3565,7 @@
         </is>
       </c>
       <c r="I30" s="38" t="n"/>
-      <c r="J30" s="27" t="inlineStr">
+      <c r="J30" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -3621,7 +3621,7 @@
           <t>BSE imaging and EDS maps (Mg, Si, Fe, Ca, S, P) on a field-emission SEM at 15 kV and 1 nA, registered to stage coordinates, each point labelled on its particle's BSE image — for both EX-CC-01 and EX-CC-02</t>
         </is>
       </c>
-      <c r="F31" s="27" t="inlineStr">
+      <c r="F31" s="30" t="inlineStr">
         <is>
           <t>Give one value; each "Sample Name" entry in a session inherits it.</t>
         </is>
@@ -3633,7 +3633,7 @@
         </is>
       </c>
       <c r="I31" s="38" t="n"/>
-      <c r="J31" s="27" t="inlineStr">
+      <c r="J31" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Sample Name".</t>
         </is>
@@ -3717,7 +3717,7 @@
           <t>JEOL</t>
         </is>
       </c>
-      <c r="F34" s="27" t="inlineStr">
+      <c r="F34" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -3729,7 +3729,7 @@
         </is>
       </c>
       <c r="I34" s="38" t="n"/>
-      <c r="J34" s="27" t="inlineStr">
+      <c r="J34" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -3785,7 +3785,7 @@
           <t>JXA-8530F Plus</t>
         </is>
       </c>
-      <c r="F35" s="27" t="inlineStr">
+      <c r="F35" s="30" t="inlineStr">
         <is>
           <t>Give one or more values for the procedure.</t>
         </is>
@@ -3797,7 +3797,7 @@
         </is>
       </c>
       <c r="I35" s="38" t="n"/>
-      <c r="J35" s="27" t="inlineStr">
+      <c r="J35" s="30" t="inlineStr">
         <is>
           <t>Give one or more values for the session.</t>
         </is>
@@ -3853,7 +3853,7 @@
           <t>Schottky field-emission</t>
         </is>
       </c>
-      <c r="F36" s="27" t="inlineStr">
+      <c r="F36" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -3865,7 +3865,7 @@
         </is>
       </c>
       <c r="I36" s="38" t="n"/>
-      <c r="J36" s="27" t="inlineStr">
+      <c r="J36" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -3921,7 +3921,7 @@
           <t>Probe for EPMA v13 (Probe Software)</t>
         </is>
       </c>
-      <c r="F37" s="27" t="inlineStr">
+      <c r="F37" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -3933,7 +3933,7 @@
         </is>
       </c>
       <c r="I37" s="38" t="n"/>
-      <c r="J37" s="27" t="inlineStr">
+      <c r="J37" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -3989,7 +3989,7 @@
           <t>Probe for EPMA v13 (point quantification); CalcImage v13 (quantitative maps); XMapTools 4 (phase classification of maps)</t>
         </is>
       </c>
-      <c r="F38" s="27" t="inlineStr">
+      <c r="F38" s="30" t="inlineStr">
         <is>
           <t>Give one or more values for the procedure.</t>
         </is>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="I38" s="38" t="n"/>
-      <c r="J38" s="27" t="inlineStr">
+      <c r="J38" s="30" t="inlineStr">
         <is>
           <t>Give one or more values for the session.</t>
         </is>
@@ -4057,7 +4057,7 @@
           <t>Five JEOL spectrometers: LDE1/TAP (Sp1); TAP/PETJ (Sp2); PETJ/LIF (Sp3); PETH/LIFH (Sp4); LIF/PETL (Sp5)</t>
         </is>
       </c>
-      <c r="F39" s="27" t="inlineStr">
+      <c r="F39" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -4069,7 +4069,7 @@
         </is>
       </c>
       <c r="I39" s="38" t="n"/>
-      <c r="J39" s="27" t="inlineStr">
+      <c r="J39" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -4125,7 +4125,7 @@
           <t>Integrated silicon drift detector: 30 mm² active area, ultra-thin polymer window, 40° take-off angle</t>
         </is>
       </c>
-      <c r="F40" s="27" t="inlineStr">
+      <c r="F40" s="30" t="inlineStr">
         <is>
           <t>Give one or more values for the procedure.</t>
         </is>
@@ -4137,7 +4137,7 @@
         </is>
       </c>
       <c r="I40" s="38" t="n"/>
-      <c r="J40" s="27" t="inlineStr">
+      <c r="J40" s="30" t="inlineStr">
         <is>
           <t>Give one or more values for the session.</t>
         </is>
@@ -4221,7 +4221,7 @@
           <t>EDS point analysis; EDS mapping; WDS point analysis; WDS mapping</t>
         </is>
       </c>
-      <c r="F43" s="27" t="inlineStr">
+      <c r="F43" s="30" t="inlineStr">
         <is>
           <t>Give one or more values for the procedure.</t>
         </is>
@@ -4233,7 +4233,7 @@
         </is>
       </c>
       <c r="I43" s="38" t="n"/>
-      <c r="J43" s="27" t="inlineStr">
+      <c r="J43" s="30" t="inlineStr">
         <is>
           <t>Give one or more values for the session.</t>
         </is>
@@ -4289,7 +4289,7 @@
           <t>Focused for silicate minerals, oxides and sulfides; defocused for phosphates; rastered for carbonates</t>
         </is>
       </c>
-      <c r="F44" s="27" t="inlineStr">
+      <c r="F44" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Material".</t>
         </is>
@@ -4301,7 +4301,7 @@
         </is>
       </c>
       <c r="I44" s="38" t="n"/>
-      <c r="J44" s="27" t="inlineStr">
+      <c r="J44" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Material".</t>
         </is>
@@ -4357,7 +4357,7 @@
           <t>15 kV (the laboratory's standard operating voltage)</t>
         </is>
       </c>
-      <c r="F45" s="27" t="inlineStr">
+      <c r="F45" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -4369,7 +4369,7 @@
         </is>
       </c>
       <c r="I45" s="38" t="n"/>
-      <c r="J45" s="27" t="inlineStr">
+      <c r="J45" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -4425,7 +4425,7 @@
           <t>20 nA for silicate minerals, oxides and sulfides; 8 nA for phosphates; 4 nA for carbonates</t>
         </is>
       </c>
-      <c r="F46" s="27" t="inlineStr">
+      <c r="F46" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Material".</t>
         </is>
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="I46" s="38" t="n"/>
-      <c r="J46" s="27" t="inlineStr">
+      <c r="J46" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Material".</t>
         </is>
@@ -4493,7 +4493,7 @@
           <t>1 µm (focused) for silicate minerals, oxides and sulfides; 5 µm (defocused) for phosphates; focused within the raster for carbonates</t>
         </is>
       </c>
-      <c r="F47" s="27" t="inlineStr">
+      <c r="F47" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Material".</t>
         </is>
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="I47" s="38" t="n"/>
-      <c r="J47" s="27" t="inlineStr">
+      <c r="J47" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Material".</t>
         </is>
@@ -4561,7 +4561,7 @@
           <t>5 × 5 µm for carbonates</t>
         </is>
       </c>
-      <c r="F48" s="27" t="inlineStr">
+      <c r="F48" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Material".</t>
         </is>
@@ -4573,7 +4573,7 @@
         </is>
       </c>
       <c r="I48" s="38" t="n"/>
-      <c r="J48" s="27" t="inlineStr">
+      <c r="J48" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Material".</t>
         </is>
@@ -4629,7 +4629,7 @@
           <t>Defocused beam for phosphates; rastered beam for carbonates; Na, K, F and Cl measured in the first acquisition pass on every point</t>
         </is>
       </c>
-      <c r="F49" s="27" t="inlineStr">
+      <c r="F49" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Material".</t>
         </is>
@@ -4641,7 +4641,7 @@
         </is>
       </c>
       <c r="I49" s="38" t="n"/>
-      <c r="J49" s="27" t="inlineStr">
+      <c r="J49" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Material".</t>
         </is>
@@ -4697,7 +4697,7 @@
           <t>Focused, for maps M1 and M2</t>
         </is>
       </c>
-      <c r="F50" s="27" t="inlineStr">
+      <c r="F50" s="30" t="inlineStr">
         <is>
           <t>Give one value; each "Sampling Unit Name" entry in a session inherits it.</t>
         </is>
@@ -4709,7 +4709,7 @@
         </is>
       </c>
       <c r="I50" s="38" t="n"/>
-      <c r="J50" s="27" t="inlineStr">
+      <c r="J50" s="30" t="inlineStr">
         <is>
           <t>For each "Sample Name", give one value for each of its "Sampling Unit Name" entries.</t>
         </is>
@@ -4765,7 +4765,7 @@
           <t>50 nA, for maps M1 and M2</t>
         </is>
       </c>
-      <c r="F51" s="27" t="inlineStr">
+      <c r="F51" s="30" t="inlineStr">
         <is>
           <t>Give one value; each "Sampling Unit Name" entry in a session inherits it.</t>
         </is>
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="I51" s="38" t="n"/>
-      <c r="J51" s="27" t="inlineStr">
+      <c r="J51" s="30" t="inlineStr">
         <is>
           <t>For each "Sample Name", give one value for each of its "Sampling Unit Name" entries.</t>
         </is>
@@ -4833,7 +4833,7 @@
           <t>1 µm (focused), for maps M1 and M2</t>
         </is>
       </c>
-      <c r="F52" s="27" t="inlineStr">
+      <c r="F52" s="30" t="inlineStr">
         <is>
           <t>Give one value; each "Sampling Unit Name" entry in a session inherits it.</t>
         </is>
@@ -4845,7 +4845,7 @@
         </is>
       </c>
       <c r="I52" s="38" t="n"/>
-      <c r="J52" s="27" t="inlineStr">
+      <c r="J52" s="30" t="inlineStr">
         <is>
           <t>For each "Sample Name", give one value for each of its "Sampling Unit Name" entries.</t>
         </is>
@@ -4901,7 +4901,7 @@
           <t>Beam current measured with the Faraday cup before each point and at the start of each map line, intensities normalised to it; primary standards re-measured at the start and end of the session, drift interpolated linearly with time</t>
         </is>
       </c>
-      <c r="F53" s="27" t="inlineStr">
+      <c r="F53" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -4913,7 +4913,7 @@
         </is>
       </c>
       <c r="I53" s="38" t="n"/>
-      <c r="J53" s="27" t="inlineStr">
+      <c r="J53" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -4969,7 +4969,7 @@
           <t>Si, Ti, Al, Cr, Fe, Mn, Mg, Ca, Na, K, P, S, F, Cl, Ni, Co, O, C (18 elements)</t>
         </is>
       </c>
-      <c r="F54" s="27" t="inlineStr">
+      <c r="F54" s="30" t="inlineStr">
         <is>
           <t>List the elements the procedure determines.</t>
         </is>
@@ -4981,7 +4981,7 @@
         </is>
       </c>
       <c r="I54" s="38" t="n"/>
-      <c r="J54" s="27" t="inlineStr">
+      <c r="J54" s="30" t="inlineStr">
         <is>
           <t>List the elements the procedure determines.</t>
         </is>
@@ -5037,7 +5037,7 @@
           <t>Si, Mg, Fe, Ca, S (EDS); Ti, Al, Cr, Mn, Na, K, P, F, Cl, Ni, Co (WDS); Zn (WDS, only to correct Zn Lα on Na Kα)</t>
         </is>
       </c>
-      <c r="F55" s="27" t="inlineStr">
+      <c r="F55" s="30" t="inlineStr">
         <is>
           <t>List each monitored element, grouped under the "Target Species" it serves (some serve none).</t>
         </is>
@@ -5049,7 +5049,7 @@
         </is>
       </c>
       <c r="I55" s="38" t="n"/>
-      <c r="J55" s="27" t="inlineStr">
+      <c r="J55" s="30" t="inlineStr">
         <is>
           <t>List each monitored element, grouped under the "Target Species" it serves (some serve none).</t>
         </is>
@@ -5105,7 +5105,7 @@
           <t>SiO₂, TiO₂, Al₂O₃, Cr₂O₃, FeO (total Fe), MnO, MgO, CaO, Na₂O, K₂O, P₂O₅, NiO, CoO in wt%; S, F, Cl in wt%; O equivalent of F and Cl; CO₂ by stoichiometry; totals; structural formulas in apfu; element maps in wt% per pixel; phase map; modal abundance in area %</t>
         </is>
       </c>
-      <c r="F56" s="27" t="inlineStr">
+      <c r="F56" s="30" t="inlineStr">
         <is>
           <t>List every quantity reported, with its unit.</t>
         </is>
@@ -5117,7 +5117,7 @@
         </is>
       </c>
       <c r="I56" s="38" t="n"/>
-      <c r="J56" s="27" t="inlineStr">
+      <c r="J56" s="30" t="inlineStr">
         <is>
           <t>List every quantity reported, with its unit.</t>
         </is>
@@ -5173,7 +5173,7 @@
           <t>EDS for Si, Mg, Fe, Ca, S; WDS for Ti, Al, Cr, Mn, Na, K, P, F, Cl, Ni, Co and for Zn (interference monitor)</t>
         </is>
       </c>
-      <c r="F57" s="27" t="inlineStr">
+      <c r="F57" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -5185,7 +5185,7 @@
         </is>
       </c>
       <c r="I57" s="38" t="n"/>
-      <c r="J57" s="27" t="inlineStr">
+      <c r="J57" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -5241,7 +5241,7 @@
           <t>Kα for every monitored element</t>
         </is>
       </c>
-      <c r="F58" s="27" t="inlineStr">
+      <c r="F58" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -5253,7 +5253,7 @@
         </is>
       </c>
       <c r="I58" s="38" t="n"/>
-      <c r="J58" s="27" t="inlineStr">
+      <c r="J58" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -5309,7 +5309,7 @@
           <t>LDE1 for F; TAP for Na, Al; PETJ for K, P, Ti; PETH for Cl; LIF for Zn, Mn, Co; LIFH for Cr; LIFH + LIF for Ni</t>
         </is>
       </c>
-      <c r="F59" s="27" t="inlineStr">
+      <c r="F59" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -5321,7 +5321,7 @@
         </is>
       </c>
       <c r="I59" s="38" t="n"/>
-      <c r="J59" s="27" t="inlineStr">
+      <c r="J59" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -5377,7 +5377,7 @@
           <t>Sp1 for F, Al; Sp2 for Na, P; Sp3 for K, Ti, Co; Sp4 for Cl, Cr; Sp5 for Zn, Mn; Sp4 + Sp5 for Ni (intensities aggregated)</t>
         </is>
       </c>
-      <c r="F60" s="27" t="inlineStr">
+      <c r="F60" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -5389,7 +5389,7 @@
         </is>
       </c>
       <c r="I60" s="38" t="n"/>
-      <c r="J60" s="27" t="inlineStr">
+      <c r="J60" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -5445,7 +5445,7 @@
           <t>Pass 1 for F, Na, K, Cl, Zn; pass 2 for Al, P, Ti, Cr, Mn; pass 3 for Co, Ni</t>
         </is>
       </c>
-      <c r="F61" s="27" t="inlineStr">
+      <c r="F61" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -5457,7 +5457,7 @@
         </is>
       </c>
       <c r="I61" s="38" t="n"/>
-      <c r="J61" s="27" t="inlineStr">
+      <c r="J61" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -5513,7 +5513,7 @@
           <t>Low-pressure P10 gas-flow counter for Sp1 and Sp2 (F, Al, Na, P); sealed Xe counter for Sp3–Sp5 (K, Ti, Co, Cl, Cr, Zn, Mn, Ni)</t>
         </is>
       </c>
-      <c r="F62" s="27" t="inlineStr">
+      <c r="F62" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -5525,7 +5525,7 @@
         </is>
       </c>
       <c r="I62" s="38" t="n"/>
-      <c r="J62" s="27" t="inlineStr">
+      <c r="J62" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -5581,7 +5581,7 @@
           <t>Differential for F, Na; integral for all other elements</t>
         </is>
       </c>
-      <c r="F63" s="27" t="inlineStr">
+      <c r="F63" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -5593,7 +5593,7 @@
         </is>
       </c>
       <c r="I63" s="38" t="n"/>
-      <c r="J63" s="27" t="inlineStr">
+      <c r="J63" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -5649,7 +5649,7 @@
           <t>20 s for F, Cl, Al, P; 10 s for Na, K, Zn; 30 s for Ti, Cr, Mn; 60 s for Co, Ni (40 s in the registered procedure)</t>
         </is>
       </c>
-      <c r="F64" s="27" t="inlineStr">
+      <c r="F64" s="30" t="inlineStr">
         <is>
           <t>For each "Target Material", give one value for each "Monitored Element".</t>
         </is>
@@ -5661,7 +5661,7 @@
         </is>
       </c>
       <c r="I64" s="38" t="n"/>
-      <c r="J64" s="27" t="inlineStr">
+      <c r="J64" s="30" t="inlineStr">
         <is>
           <t>For each "Target Material", give one value for each "Monitored Element".</t>
         </is>
@@ -5717,7 +5717,7 @@
           <t>20 s for F, Cl, Al, P; 10 s for Na, K, Zn; 30 s for Ti, Cr, Mn; 60 s for Co, Ni (total of both positions)</t>
         </is>
       </c>
-      <c r="F65" s="27" t="inlineStr">
+      <c r="F65" s="30" t="inlineStr">
         <is>
           <t>For each "Target Material", give one value for each "Monitored Element".</t>
         </is>
@@ -5729,7 +5729,7 @@
         </is>
       </c>
       <c r="I65" s="38" t="n"/>
-      <c r="J65" s="27" t="inlineStr">
+      <c r="J65" s="30" t="inlineStr">
         <is>
           <t>For each "Target Material", give one value for each "Monitored Element".</t>
         </is>
@@ -5785,7 +5785,7 @@
           <t>−3.2 / +4.5 mm for F; −4.0 / +4.0 mm for Na, P; −4.5 / +4.5 mm for K; −3.0 / +3.0 mm for Cl, Cr, Ni; −3.5 / +3.5 mm for Zn, Al, Mn; −5.0 / +5.0 mm for Ti; −2.5 / +3.5 mm for Co</t>
         </is>
       </c>
-      <c r="F66" s="27" t="inlineStr">
+      <c r="F66" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -5797,7 +5797,7 @@
         </is>
       </c>
       <c r="I66" s="38" t="n"/>
-      <c r="J66" s="27" t="inlineStr">
+      <c r="J66" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -5853,7 +5853,7 @@
           <t>30 s per point</t>
         </is>
       </c>
-      <c r="F67" s="27" t="inlineStr">
+      <c r="F67" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -5865,7 +5865,7 @@
         </is>
       </c>
       <c r="I67" s="38" t="n"/>
-      <c r="J67" s="27" t="inlineStr">
+      <c r="J67" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -5921,7 +5921,7 @@
           <t>Point spectra; spectrum images (full spectrum at every pixel); no line scans</t>
         </is>
       </c>
-      <c r="F68" s="27" t="inlineStr">
+      <c r="F68" s="30" t="inlineStr">
         <is>
           <t>Give one or more values for the procedure.</t>
         </is>
@@ -5933,7 +5933,7 @@
         </is>
       </c>
       <c r="I68" s="38" t="n"/>
-      <c r="J68" s="27" t="inlineStr">
+      <c r="J68" s="30" t="inlineStr">
         <is>
           <t>Give one or more values for the session.</t>
         </is>
@@ -5989,7 +5989,7 @@
           <t>30 ms per pixel for Na, Al, P, Cr, Ni (WDS) and for the EDS spectrum image</t>
         </is>
       </c>
-      <c r="F69" s="27" t="inlineStr">
+      <c r="F69" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -6001,7 +6001,7 @@
         </is>
       </c>
       <c r="I69" s="38" t="n"/>
-      <c r="J69" s="27" t="inlineStr">
+      <c r="J69" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -6057,7 +6057,7 @@
           <t>2 µm in both X and Y</t>
         </is>
       </c>
-      <c r="F70" s="27" t="inlineStr">
+      <c r="F70" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -6069,7 +6069,7 @@
         </is>
       </c>
       <c r="I70" s="38" t="n"/>
-      <c r="J70" s="27" t="inlineStr">
+      <c r="J70" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -6125,7 +6125,7 @@
           <t>512 × 512 pixels for M1; 384 × 256 pixels for M2</t>
         </is>
       </c>
-      <c r="F71" s="27" t="inlineStr">
+      <c r="F71" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -6137,7 +6137,7 @@
         </is>
       </c>
       <c r="I71" s="38" t="n"/>
-      <c r="J71" s="27" t="inlineStr">
+      <c r="J71" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -6193,7 +6193,7 @@
           <t>1.024 × 1.024 mm for M1; 0.768 × 0.512 mm for M2</t>
         </is>
       </c>
-      <c r="F72" s="27" t="inlineStr">
+      <c r="F72" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -6205,7 +6205,7 @@
         </is>
       </c>
       <c r="I72" s="38" t="n"/>
-      <c r="J72" s="27" t="inlineStr">
+      <c r="J72" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -6261,7 +6261,7 @@
           <t>Stage scan with the beam held fixed</t>
         </is>
       </c>
-      <c r="F73" s="27" t="inlineStr">
+      <c r="F73" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -6273,7 +6273,7 @@
         </is>
       </c>
       <c r="I73" s="38" t="n"/>
-      <c r="J73" s="27" t="inlineStr">
+      <c r="J73" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -6357,7 +6357,7 @@
           <t>Armstrong/Love–Scott φ(ρz) matrix correction (Armstrong 1995) in Probe for EPMA; applied pixel by pixel in CalcImage for maps</t>
         </is>
       </c>
-      <c r="F76" s="27" t="inlineStr">
+      <c r="F76" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -6369,7 +6369,7 @@
         </is>
       </c>
       <c r="I76" s="38" t="n"/>
-      <c r="J76" s="27" t="inlineStr">
+      <c r="J76" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -6425,7 +6425,7 @@
           <t>FFAST (Chantler et al. 2005)</t>
         </is>
       </c>
-      <c r="F77" s="27" t="inlineStr">
+      <c r="F77" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -6437,7 +6437,7 @@
         </is>
       </c>
       <c r="I77" s="38" t="n"/>
-      <c r="J77" s="27" t="inlineStr">
+      <c r="J77" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -6493,7 +6493,7 @@
           <t>Removed by filter fitting for Si, Mg, Fe, Ca, S (EDS); two-point off-peak, linear for WDS elements in points, exponential for F; MAN calibration (Donovan and Tingle 1996) for WDS maps</t>
         </is>
       </c>
-      <c r="F78" s="27" t="inlineStr">
+      <c r="F78" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -6505,7 +6505,7 @@
         </is>
       </c>
       <c r="I78" s="38" t="n"/>
-      <c r="J78" s="27" t="inlineStr">
+      <c r="J78" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Monitored Element".</t>
         </is>
@@ -6561,7 +6561,7 @@
           <t>Linear for Na; exponential for F (in apatite); none for other elements</t>
         </is>
       </c>
-      <c r="F79" s="27" t="inlineStr">
+      <c r="F79" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Species".</t>
         </is>
@@ -6573,7 +6573,7 @@
         </is>
       </c>
       <c r="I79" s="38" t="n"/>
-      <c r="J79" s="27" t="inlineStr">
+      <c r="J79" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Species".</t>
         </is>
@@ -6629,7 +6629,7 @@
           <t>Directly from measured intensities for every measured element; by stoichiometry from cation valences for O; as CO₂ by stoichiometry for C (carbonates only); OH in apatite by difference, F + Cl + OH = 1 apfu (Ketcham 2015)</t>
         </is>
       </c>
-      <c r="F80" s="27" t="inlineStr">
+      <c r="F80" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Species".</t>
         </is>
@@ -6641,7 +6641,7 @@
         </is>
       </c>
       <c r="I80" s="38" t="n"/>
-      <c r="J80" s="27" t="inlineStr">
+      <c r="J80" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Species".</t>
         </is>
@@ -6697,7 +6697,7 @@
           <t>Oxygen equivalent of F and Cl subtracted from the total (apatite)</t>
         </is>
       </c>
-      <c r="F81" s="27" t="inlineStr">
+      <c r="F81" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -6709,7 +6709,7 @@
         </is>
       </c>
       <c r="I81" s="38" t="n"/>
-      <c r="J81" s="27" t="inlineStr">
+      <c r="J81" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -6765,7 +6765,7 @@
           <t>Logarithmic expression; spectrometer-specific constants of 1.1–1.5 µs</t>
         </is>
       </c>
-      <c r="F82" s="27" t="inlineStr">
+      <c r="F82" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -6777,7 +6777,7 @@
         </is>
       </c>
       <c r="I82" s="38" t="n"/>
-      <c r="J82" s="27" t="inlineStr">
+      <c r="J82" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -6833,7 +6833,7 @@
           <t>Filter fitting: a top-hat filter followed by least-squares fitting to measured standard spectra</t>
         </is>
       </c>
-      <c r="F83" s="27" t="inlineStr">
+      <c r="F83" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -6845,7 +6845,7 @@
         </is>
       </c>
       <c r="I83" s="38" t="n"/>
-      <c r="J83" s="27" t="inlineStr">
+      <c r="J83" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -6901,7 +6901,7 @@
           <t>Apparent concentration measured on Ni- and Co-free synthetic forsterite subtracted, for Ni and Co; none for other elements</t>
         </is>
       </c>
-      <c r="F84" s="27" t="inlineStr">
+      <c r="F84" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Species".</t>
         </is>
@@ -6913,7 +6913,7 @@
         </is>
       </c>
       <c r="I84" s="38" t="n"/>
-      <c r="J84" s="27" t="inlineStr">
+      <c r="J84" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Species".</t>
         </is>
@@ -6969,7 +6969,7 @@
           <t>Structural formulas normalised to a fixed anion basis: 4 O for olivine and spinels, 6 O for pyroxene and dolomite, 3 O for calcite, 13 anions for apatite (Ketcham 2015); none for other reported variables</t>
         </is>
       </c>
-      <c r="F85" s="27" t="inlineStr">
+      <c r="F85" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Reported Variable".</t>
         </is>
@@ -6981,7 +6981,7 @@
         </is>
       </c>
       <c r="I85" s="38" t="n"/>
-      <c r="J85" s="27" t="inlineStr">
+      <c r="J85" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Reported Variable".</t>
         </is>
@@ -7037,7 +7037,7 @@
           <t>None, for every reported variable (concentrations from k-ratios against the primary standards)</t>
         </is>
       </c>
-      <c r="F86" s="27" t="inlineStr">
+      <c r="F86" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Reported Variable".</t>
         </is>
@@ -7049,7 +7049,7 @@
         </is>
       </c>
       <c r="I86" s="38" t="n"/>
-      <c r="J86" s="27" t="inlineStr">
+      <c r="J86" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Reported Variable".</t>
         </is>
@@ -7105,7 +7105,7 @@
           <t>35 ± 9 µg/g for Ni; 22 ± 8 µg/g for Co (n = 5)</t>
         </is>
       </c>
-      <c r="F87" s="27" t="inlineStr">
+      <c r="F87" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -7117,7 +7117,7 @@
         </is>
       </c>
       <c r="I87" s="38" t="n"/>
-      <c r="J87" s="27" t="inlineStr">
+      <c r="J87" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Species".</t>
         </is>
@@ -7173,7 +7173,7 @@
           <t>Rules: totals 98.5–101.5 wt% (silicates, oxides, sulfides), 96.0–101.5 (apatite), 98.0–102.0 (carbonates); cation sum within ±0.03 apfu; no overlap with a second phase; beam drift under 1%. Outcome: 53 points acquired, 45 included; excluded P3-02 and P3-05 from apatite in EX-CC-01 and P1-03, P1-07 from dolomite in EX-CC-02 (totals), P2-07 and P2-09 from pyrrhotite in EX-CC-01 and P1-16 from calcite in EX-CC-02 (overlap), P2-05 from olivine in EX-CC-02 (drift)</t>
         </is>
       </c>
-      <c r="F88" s="27" t="inlineStr">
+      <c r="F88" s="30" t="inlineStr">
         <is>
           <t>Give one value; each "Combined Result" entry in a session inherits it.</t>
         </is>
@@ -7185,7 +7185,7 @@
         </is>
       </c>
       <c r="I88" s="38" t="n"/>
-      <c r="J88" s="27" t="inlineStr">
+      <c r="J88" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Combined Result".</t>
         </is>
@@ -7241,7 +7241,7 @@
           <t>Arithmetic mean of the included points, per phase within each sample, for every oxide and element concentration; maps and structural formulas not combined</t>
         </is>
       </c>
-      <c r="F89" s="27" t="inlineStr">
+      <c r="F89" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Reported Variable".</t>
         </is>
@@ -7253,7 +7253,7 @@
         </is>
       </c>
       <c r="I89" s="38" t="n"/>
-      <c r="J89" s="27" t="inlineStr">
+      <c r="J89" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Reported Variable".</t>
         </is>
@@ -7309,7 +7309,7 @@
           <t>Olivine in EX-CC-01 (P1-01–P1-08); pyroxene in EX-CC-01 (P1-09–P1-12); magnetite in EX-CC-01 (P2-01–P2-06); pyrrhotite in EX-CC-01 (P2-07–P2-11); apatite in EX-CC-01 (P3-01–P3-06); dolomite in EX-CC-02 (P1-01–P1-10); calcite in EX-CC-02 (P1-11–P1-16); olivine in EX-CC-02 (P2-01–P2-08)</t>
         </is>
       </c>
-      <c r="F90" s="27" t="inlineStr">
+      <c r="F90" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -7321,7 +7321,7 @@
         </is>
       </c>
       <c r="I90" s="38" t="n"/>
-      <c r="J90" s="27" t="inlineStr">
+      <c r="J90" s="30" t="inlineStr">
         <is>
           <t>List every reported value that combines several individual results, saying what each combines.</t>
         </is>
@@ -7377,7 +7377,7 @@
           <t>IUPAC 2021 standard atomic weights (Prohaska et al. 2022)</t>
         </is>
       </c>
-      <c r="F91" s="27" t="inlineStr">
+      <c r="F91" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -7389,7 +7389,7 @@
         </is>
       </c>
       <c r="I91" s="38" t="n"/>
-      <c r="J91" s="27" t="inlineStr">
+      <c r="J91" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -7473,7 +7473,7 @@
           <t>Springwater olivine USNM 2566 for Si, Mg; Rockport fayalite USNM 85276 for Fe; diopside USNM 117733 for Ca; dolomite USNM 10057 for Ca, Mg in carbonates; synthetic FeS for S; synthetic SrF₂ for F; Amelia albite for Na; microcline USNM 143966 for K; scapolite USNM R6600-1 for Cl; anorthite USNM 137041 for Al; Wilberforce fluorapatite for P; ilmenite USNM 96189 for Ti; synthetic Cr₂O₃ for Cr; rhodonite for Mn; Co metal for Co; Ni metal for Ni; synthetic ZnS for Zn (Smithsonian values: Jarosewich et al. 1980)</t>
         </is>
       </c>
-      <c r="F94" s="27" t="inlineStr">
+      <c r="F94" s="30" t="inlineStr">
         <is>
           <t>For each "Target Material", give one value for each "Target Species".</t>
         </is>
@@ -7485,7 +7485,7 @@
         </is>
       </c>
       <c r="I94" s="38" t="n"/>
-      <c r="J94" s="27" t="inlineStr">
+      <c r="J94" s="30" t="inlineStr">
         <is>
           <t>For each "Target Material", give one value for each "Target Species".</t>
         </is>
@@ -7541,7 +7541,7 @@
           <t>San Carlos olivine USNM 111312/444; Kakanui augite USNM 122142; Durango apatite USNM 104021; chromite USNM 117075; calcite USNM 136321 (accepted values: Jarosewich et al. 1980)</t>
         </is>
       </c>
-      <c r="F95" s="27" t="inlineStr">
+      <c r="F95" s="30" t="inlineStr">
         <is>
           <t>List the secondary reference materials run as unknowns.</t>
         </is>
@@ -7553,7 +7553,7 @@
         </is>
       </c>
       <c r="I95" s="38" t="n"/>
-      <c r="J95" s="27" t="inlineStr">
+      <c r="J95" s="30" t="inlineStr">
         <is>
           <t>List the secondary reference materials run as unknowns.</t>
         </is>
@@ -7609,7 +7609,7 @@
           <t>Yes for Co (Fe Kβ on Co Kα), Mn (Cr Kβ on Mn Kα) and Na (Zn Lα on Na Kα), quantitative and iterated with the matrix correction; no for all other elements</t>
         </is>
       </c>
-      <c r="F96" s="27" t="inlineStr">
+      <c r="F96" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Species".</t>
         </is>
@@ -7621,7 +7621,7 @@
         </is>
       </c>
       <c r="I96" s="38" t="n"/>
-      <c r="J96" s="27" t="inlineStr">
+      <c r="J96" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Species".</t>
         </is>
@@ -7677,7 +7677,7 @@
           <t>Fe for Co; Cr for Mn; Zn for Na</t>
         </is>
       </c>
-      <c r="F97" s="27" t="inlineStr">
+      <c r="F97" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Species".</t>
         </is>
@@ -7689,7 +7689,7 @@
         </is>
       </c>
       <c r="I97" s="38" t="n"/>
-      <c r="J97" s="27" t="inlineStr">
+      <c r="J97" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Species".</t>
         </is>
@@ -7745,7 +7745,7 @@
           <t>Co-free Rockport fayalite for Co; Mn-free synthetic Cr₂O₃ for Mn; Na-free synthetic ZnS for Na</t>
         </is>
       </c>
-      <c r="F98" s="27" t="inlineStr">
+      <c r="F98" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Species".</t>
         </is>
@@ -7757,7 +7757,7 @@
         </is>
       </c>
       <c r="I98" s="38" t="n"/>
-      <c r="J98" s="27" t="inlineStr">
+      <c r="J98" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Target Species".</t>
         </is>
@@ -7813,7 +7813,7 @@
           <t>Points (wt%): 0.11 SiO₂, 0.09 MgO, 0.14 FeO, 0.10 CaO, 0.08 S (EDS); 0.055 F, 0.018 Na₂O, 0.009 K₂O, 0.010 Cl, 0.012 Al₂O₃, 0.020 P₂O₅, 0.015 TiO₂, 0.018 Cr₂O₃, 0.016 MnO, 0.010 CoO, 0.008 NiO (WDS). Maps: about 0.3 wt% per pixel (WDS), 0.7 wt% (EDS)</t>
         </is>
       </c>
-      <c r="F99" s="27" t="inlineStr">
+      <c r="F99" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Reported Variable".</t>
         </is>
@@ -7825,7 +7825,7 @@
         </is>
       </c>
       <c r="I99" s="38" t="n"/>
-      <c r="J99" s="27" t="inlineStr">
+      <c r="J99" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Reported Variable".</t>
         </is>
@@ -7881,7 +7881,7 @@
           <t>3σ of the background counts, for every reported variable</t>
         </is>
       </c>
-      <c r="F100" s="27" t="inlineStr">
+      <c r="F100" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Reported Variable".</t>
         </is>
@@ -7893,7 +7893,7 @@
         </is>
       </c>
       <c r="I100" s="38" t="n"/>
-      <c r="J100" s="27" t="inlineStr">
+      <c r="J100" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Reported Variable".</t>
         </is>
@@ -7949,7 +7949,7 @@
           <t>0.4–0.7% for oxides above 10 wt%; 0.9–1.6% for FeO and Al₂O₃; 2–4% for TiO₂, Na₂O, F and Cl; 4% for NiO in San Carlos olivine (1σ RSD; San Carlos olivine n = 9, Kakanui augite n = 6, Durango apatite n = 6, chromite n = 5, calcite n = 6)</t>
         </is>
       </c>
-      <c r="F101" s="27" t="inlineStr">
+      <c r="F101" s="30" t="inlineStr">
         <is>
           <t>For each "Secondary Reference Material", give one value for each "Reported Variable".</t>
         </is>
@@ -7961,7 +7961,7 @@
         </is>
       </c>
       <c r="I101" s="38" t="n"/>
-      <c r="J101" s="27" t="inlineStr">
+      <c r="J101" s="30" t="inlineStr">
         <is>
           <t>For each "Secondary Reference Material", give one value for each "Reported Variable".</t>
         </is>
@@ -8017,7 +8017,7 @@
           <t>Within ±1.2% relative for all major oxides; within ±2.6% for minor oxides and halogens</t>
         </is>
       </c>
-      <c r="F102" s="27" t="inlineStr">
+      <c r="F102" s="30" t="inlineStr">
         <is>
           <t>For each "Secondary Reference Material", give one value for each "Reported Variable".</t>
         </is>
@@ -8029,7 +8029,7 @@
         </is>
       </c>
       <c r="I102" s="38" t="n"/>
-      <c r="J102" s="27" t="inlineStr">
+      <c r="J102" s="30" t="inlineStr">
         <is>
           <t>For each "Secondary Reference Material", give one value for each "Reported Variable".</t>
         </is>
@@ -8085,7 +8085,7 @@
           <t>1σ from counting statistics on the peak and on any subtracted background or blank, for every analysis and every reported variable; in olivine about 0.5% relative for SiO₂ and MgO, about 10% for NiO at 0.03 wt%</t>
         </is>
       </c>
-      <c r="F103" s="27" t="inlineStr">
+      <c r="F103" s="30" t="inlineStr">
         <is>
           <t>Give one value for each "Reported Variable".</t>
         </is>
@@ -8097,7 +8097,7 @@
         </is>
       </c>
       <c r="I103" s="38" t="n"/>
-      <c r="J103" s="27" t="inlineStr">
+      <c r="J103" s="30" t="inlineStr">
         <is>
           <t>For each "Sample Name", give one value for every "Reported Variable" at every "Sampling Unit Name" entry.</t>
         </is>
@@ -8153,7 +8153,7 @@
           <t>18–26% during point analysis; 24–31% during spectrum imaging</t>
         </is>
       </c>
-      <c r="F104" s="27" t="inlineStr">
+      <c r="F104" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -8165,7 +8165,7 @@
         </is>
       </c>
       <c r="I104" s="38" t="n"/>
-      <c r="J104" s="27" t="inlineStr">
+      <c r="J104" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>
@@ -8221,7 +8221,7 @@
           <t>MSWD of the included points about the mean: for olivine in EX-CC-01, 0.9 for NiO to 2.3 for CaO, and 4.6 for FeO (Fe–Mg zoning); likewise for every other combined result</t>
         </is>
       </c>
-      <c r="F105" s="27" t="inlineStr">
+      <c r="F105" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -8233,7 +8233,7 @@
         </is>
       </c>
       <c r="I105" s="38" t="n"/>
-      <c r="J105" s="27" t="inlineStr">
+      <c r="J105" s="30" t="inlineStr">
         <is>
           <t>For each "Combined Result", give one value for each "Reported Variable".</t>
         </is>
@@ -8289,7 +8289,7 @@
           <t>Standard error of the mean (1 s.d./√n): for olivine in EX-CC-01, 0.08 wt% for SiO₂, 0.12 for MgO, 0.04 for FeO; likewise for every other combined result</t>
         </is>
       </c>
-      <c r="F106" s="27" t="inlineStr">
+      <c r="F106" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -8301,7 +8301,7 @@
         </is>
       </c>
       <c r="I106" s="38" t="n"/>
-      <c r="J106" s="27" t="inlineStr">
+      <c r="J106" s="30" t="inlineStr">
         <is>
           <t>For each "Combined Result", give one value for each "Reported Variable".</t>
         </is>
@@ -8357,7 +8357,7 @@
           <t>Particle P2 of EX-CC-02 partly plucked during ion polishing; its analyses lie on the remaining fragment. No other anomalies, instrument modifications or departures</t>
         </is>
       </c>
-      <c r="F107" s="27" t="inlineStr">
+      <c r="F107" s="30" t="inlineStr">
         <is>
           <t>Give one value for the procedure.</t>
         </is>
@@ -8369,7 +8369,7 @@
         </is>
       </c>
       <c r="I107" s="38" t="n"/>
-      <c r="J107" s="27" t="inlineStr">
+      <c r="J107" s="30" t="inlineStr">
         <is>
           <t>Give one value for the session.</t>
         </is>

</xml_diff>